<commit_message>
Daily EOD data and reports for 2026-10-30
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261030.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261030.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.602</v>
+        <v>1.605</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.038</v>
+        <v>-0.035</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-2.13%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>245395.96</v>
+        <v>245855.51</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-5820.88</v>
+        <v>-5361.33</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.515</v>
+        <v>2.54</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.005</v>
+        <v>0.03</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.20%</t>
+          <t>1.20%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>176050</v>
+        <v>177800</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>350</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>57.39</v>
+        <v>57.56</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.13</v>
+        <v>0.04</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.23%</t>
+          <t>0.07%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>459120</v>
+        <v>460480</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-1040</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>166.86</v>
+        <v>166.72</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.47</v>
+        <v>0.33</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.805</v>
+        <v>0.79</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.015</v>
+        <v>-0.03</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.83%</t>
+          <t>-3.66%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8050</v>
+        <v>7900</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-150</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>200.035</v>
+        <v>200.73</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2.535</v>
+        <v>3.23</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.28%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>800140</v>
+        <v>802920</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>10140</v>
+        <v>12920</v>
       </c>
     </row>
     <row r="11">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>11.32</v>
+        <v>11.34</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.45</v>
+        <v>-0.43</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-3.82%</t>
+          <t>-3.65%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>34469.4</v>
+        <v>34530.3</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-1370.25</v>
+        <v>-1309.35</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.081</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.083</v>
+        <v>-0.002</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-2.41%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>762.37</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-781.2</v>
+        <v>-18.82</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>37.06</v>
+        <v>36.82</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.39</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.40%</t>
+          <t>-1.05%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.35</v>
+        <v>33.33</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.86%</t>
+          <t>1.80%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42954.8</v>
+        <v>42929.04</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>785.6799999999999</v>
+        <v>759.92</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1770974.61</v>
+        <v>1777971.67</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>513.36</v>
+        <v>7510.41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>